<commit_message>
base de datos y explciasion
</commit_message>
<xml_diff>
--- a/base de datos/diccionario de datos de BD.xlsx
+++ b/base de datos/diccionario de datos de BD.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Documents\trabajo isseg\base de datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C34B7EFC-9469-4037-B892-54D27225D97B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9E4C68A-21F0-491E-9E64-049114EDD794}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6330" yWindow="3045" windowWidth="21600" windowHeight="11295" xr2:uid="{521348AD-0B1B-488A-B674-FA16CC85AB04}"/>
   </bookViews>
@@ -468,6 +468,12 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>